<commit_message>
Sales Data Has been updated today
</commit_message>
<xml_diff>
--- a/Sales Data/SalesDatasept2026.xlsx
+++ b/Sales Data/SalesDatasept2026.xlsx
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="Sept2026" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sept2026!$A$2:$D$2</definedName>
+  </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -24,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="60">
   <si>
     <t>Sales Data of Sattvik Bhojan of Month Sept ,2026</t>
   </si>
@@ -59,9 +62,6 @@
     <t xml:space="preserve">Item </t>
   </si>
   <si>
-    <t>Online through GooglePay</t>
-  </si>
-  <si>
     <t>1 Kadahi Panner +Kadhi</t>
   </si>
   <si>
@@ -96,13 +96,124 @@
   </si>
   <si>
     <t>5 Plate of Rajma +1 Kadahi</t>
+  </si>
+  <si>
+    <t>19/9/2026</t>
+  </si>
+  <si>
+    <t>1 Plate Kadhi Chalwal</t>
+  </si>
+  <si>
+    <t>1 Bowl of kadhi</t>
+  </si>
+  <si>
+    <t>18/9/2026</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>12 Chapati +1 kadahi Panner +1 Bowl of Rajma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/9/2026 </t>
+  </si>
+  <si>
+    <t>Kadahi Panner</t>
+  </si>
+  <si>
+    <t>Tiffin Box</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unkown </t>
+  </si>
+  <si>
+    <t>16/9/2026</t>
+  </si>
+  <si>
+    <t>ZERO SALE</t>
+  </si>
+  <si>
+    <t>NO SALE</t>
+  </si>
+  <si>
+    <t>17/9/2026</t>
+  </si>
+  <si>
+    <t>1 Chana</t>
+  </si>
+  <si>
+    <t>1 Plate of Kadhi +1Mix Veg+4 Chapati+1 Rice</t>
+  </si>
+  <si>
+    <t>Kadahi Chalwal</t>
+  </si>
+  <si>
+    <t>20/9/2026</t>
+  </si>
+  <si>
+    <t>1 Bowl of Kadhi +12 Chapati</t>
+  </si>
+  <si>
+    <t>2 Bowl of Rajma</t>
+  </si>
+  <si>
+    <t>1 Mix Veg + 1 chana</t>
+  </si>
+  <si>
+    <t>21/9/2026</t>
+  </si>
+  <si>
+    <t>22/9/2026</t>
+  </si>
+  <si>
+    <t>1 kadhi + 1 Plate of Rice+1 Mix Veg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 kadhi + 4 chapati </t>
+  </si>
+  <si>
+    <t>1 Kadhi + 6 chapati</t>
+  </si>
+  <si>
+    <t>1 Paneer Bhurji</t>
+  </si>
+  <si>
+    <t>1 Bowl of Dal+ Mix Veg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 paneer Bhurji + 8 chapati </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 paneer Bhurji </t>
+  </si>
+  <si>
+    <t>1 Kadahi Paneer + 10 Chapati</t>
+  </si>
+  <si>
+    <t>1 Mater Mushroom + 1 Mix Veg</t>
+  </si>
+  <si>
+    <t>1 mater Mushroom + 2 Chapati</t>
+  </si>
+  <si>
+    <t>1 kadahi +1 Rice +2 Chapati</t>
+  </si>
+  <si>
+    <t>1 Kadahi Panner+Kadhi+Chapati</t>
+  </si>
+  <si>
+    <t>1 Tiffin Box</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,16 +228,34 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -149,39 +278,47 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,229 +600,616 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="36.54296875" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="40.26953125" customWidth="1"/>
     <col min="3" max="3" width="13.1796875" customWidth="1"/>
     <col min="4" max="4" width="23.36328125" customWidth="1"/>
     <col min="5" max="5" width="17.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="A3" s="3">
+        <v>46304</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2">
+        <v>75</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="A4" s="3">
+        <v>46304</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="2">
+        <v>120</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3">
+      <c r="A5" s="4">
         <v>46335</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C5" s="2">
         <f>2*40</f>
         <v>80</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3">
+      <c r="D5" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
         <v>46335</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C6" s="2">
         <f>5*20</f>
         <v>100</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3">
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
         <v>46365</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C7" s="2">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="3">
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
         <v>46365</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C8" s="2">
         <f>35+40</f>
         <v>75</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>46365</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2">
+        <f>4*40</f>
+        <v>160</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>46365</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2">
+        <f>40+40</f>
+        <v>80</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>46365</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="1">
-        <f>4*40</f>
-        <v>160</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="B11" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="2">
+        <v>130</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="3">
-        <v>46365</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="1">
-        <f>40+40</f>
-        <v>80</v>
-      </c>
-      <c r="D12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="2">
+        <f>45+135</f>
+        <v>180</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="5">
-        <v>46365</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="1">
-        <v>130</v>
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2">
+        <v>150</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C15">
-        <v>150</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C14" s="2">
+        <v>270</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="28" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="2">
+        <v>400</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16">
-        <v>270</v>
-      </c>
-      <c r="D16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17">
-        <v>400</v>
-      </c>
-      <c r="D17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B16" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18">
+      <c r="C16" s="2">
         <f>6*40</f>
         <v>240</v>
       </c>
-      <c r="D18" t="s">
-        <v>21</v>
+      <c r="D16" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="9">
+        <v>40</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="2">
+        <v>235</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="2">
+        <v>50</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="2">
+        <v>150</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="2">
+        <v>135</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="2">
+        <v>45</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="2">
+        <v>40</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="12">
+        <f>40+5*12</f>
+        <v>100</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="11">
+        <v>80</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="11">
+        <v>100</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="11">
+        <v>70</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="11">
+        <v>100</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="12">
+        <f>110+5*8</f>
+        <v>150</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="11">
+        <v>110</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="12">
+        <f>135+10*5</f>
+        <v>185</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="12">
+        <f>90+40</f>
+        <v>130</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="12">
+        <f>40+35+2*5</f>
+        <v>85</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="12">
+        <v>250</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" s="12">
+        <f>90+2*5</f>
+        <v>100</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="12">
+        <f>40+35+40</f>
+        <v>115</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="12">
+        <f>40+4*5</f>
+        <v>60</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="12">
+        <f>40+5*6</f>
+        <v>70</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" s="12">
+        <v>110</v>
+      </c>
+      <c r="D40" s="12"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="12">
+        <v>70</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D2"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <conditionalFormatting sqref="A2:D2">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="0"/>
+        <color theme="5"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>